<commit_message>
Update reporting scripts and merge output; refresh ledgers and reports
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MERGE_SCRIPT/Daywize_Snapshot.xlsx
+++ b/MERGE_SCRIPT/Daywize_Snapshot.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daywize_Snapshot" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daywize_Snapshot_paper" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,14 +446,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20-Jun-2026</t>
+          <t>25-Jun-2026</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -465,11 +465,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>24-Jun-2026</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -484,14 +484,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>23-Jun-2026</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -503,19 +503,76 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>20-Jun-2026</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>19-Jun-2026</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>106</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>18-Jun-2026</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>106</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>17-Jun-2026</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B8" t="n">
         <v>97</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C8" t="n">
         <v>149</v>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update reporting scripts, ledgers, and reports
</commit_message>
<xml_diff>
--- a/MERGE_SCRIPT/Daywize_Snapshot.xlsx
+++ b/MERGE_SCRIPT/Daywize_Snapshot.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,14 +446,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>26-Jun-2026</t>
+          <t>27-Jun-2026</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>121</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -465,14 +465,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25-Jun-2026</t>
+          <t>26-Jun-2026</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -484,14 +484,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>24-Jun-2026</t>
+          <t>25-Jun-2026</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -503,14 +503,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>23-Jun-2026</t>
+          <t>24-Jun-2026</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C5" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -522,14 +522,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20-Jun-2026</t>
+          <t>23-Jun-2026</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -541,7 +541,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>20-Jun-2026</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -560,14 +560,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>19-Jun-2026</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>106</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -579,19 +579,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>18-Jun-2026</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>106</v>
+      </c>
+      <c r="C9" t="n">
+        <v>13</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>17-Jun-2026</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>97</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C10" t="n">
         <v>149</v>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>